<commit_message>
feat: FER modeli Veri Füzyonu ile optimize edildi, makale raporu ve canli_test.py eklendi
</commit_message>
<xml_diff>
--- a/deney_sonuclari.xlsx
+++ b/deney_sonuclari.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -659,6 +659,151 @@
         <v>62.73</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-03-24 11:04:55</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr"/>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Fine Tuning + Class Weights + Checkpoint</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="n">
+        <v>30</v>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="n">
+        <v>64.23999999999999</v>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="n">
+        <v>72.05</v>
+      </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="n">
+        <v>66.17</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-03-24 11:33:47</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Deeper Fine Tuning (100 Layers) + Dropout 0.3</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="n">
+        <v>26</v>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="n">
+        <v>63.69</v>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="n">
+        <v>71.52</v>
+      </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="n">
+        <v>65.90000000000001</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-03-24 12:06:05</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr"/>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>EfficientNetB0 + Class Weights + Dropout 0.4</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="n">
+        <v>29</v>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="n">
+        <v>63.53</v>
+      </c>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="n">
+        <v>70.3</v>
+      </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="n">
+        <v>65.45</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-03-24 12:34:36</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr"/>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>ResNet50V2 + Otomatik Split + Dropout 0.4</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="n">
+        <v>30</v>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="n">
+        <v>95.41</v>
+      </c>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="n">
+        <v>96.17</v>
+      </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="n">
+        <v>95.69</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-03-24 13:57:42</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr"/>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>MobileNetV2 (Canlı Optimizasyon) + Veri Füzyonu + Dropout 0.4</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="n">
+        <v>30</v>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="n">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="n">
+        <v>72.12</v>
+      </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="n">
+        <v>67.62</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>